<commit_message>
Trend : rapport PDF corrigé après vérification indépendante
- Monétaire couru en jours calendaires (au lieu de /252 sur ~261 jours) ;
  Nasdaq-100 : indice de prix jusqu'en 2002 (cours de QQQ bruités en 1999-2002).
- Exposition moyenne et coûts par an de chaque variante ; tableau des grandes
  baisses du S&P 500 avec l'indice SG Trend (vrais fonds) en regard.
- Texte : chiffres calculés plutôt qu'écrits en dur, levier par variante, années
  de crise sans sélection, situation actuelle sous les sommets, dépendance aux
  données (Carver vs 84 marchés), coûts exacts, unités en dollars, typographie.
- Excel : formats pourcentage / ratio corrects.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uj28ULkDfXKqEeuebxHWZb
</commit_message>
<xml_diff>
--- a/analyse-trend/rapport/performances_annuelles.xlsx
+++ b/analyse-trend/rapport/performances_annuelles.xlsx
@@ -10,8 +10,9 @@
     <sheet name="Années 1990-2026" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Indicateurs 1990-2026" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="CAGR par période" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Carry années 1990-2024" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Carry indicateurs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Baisses des actions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Carry années 1990-2024" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Carry indicateurs" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -482,19 +483,19 @@
         <v>1990</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>0.6801501904078722</v>
+        <v>0.6756812923669719</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>0.7158042013283801</v>
+        <v>0.7111998018952796</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>0.8266906593185785</v>
+        <v>0.8217668982345221</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>0.9636840727776113</v>
+        <v>0.9583602678167824</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>1.113519887330518</v>
+        <v>1.107785016528875</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>-0.03104820642576656</v>
@@ -503,7 +504,7 @@
         <v>-0.1041168718028905</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>0.08066065701536451</v>
+        <v>0.07774330018656528</v>
       </c>
     </row>
     <row r="3">
@@ -511,19 +512,19 @@
         <v>1991</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>0.2908407043731664</v>
+        <v>0.288408219383796</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>0.42985247461127</v>
+        <v>0.4271673153147306</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>0.5165922421573179</v>
+        <v>0.5137527916211624</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>0.7920401322007113</v>
+        <v>0.7886749332260363</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>0.7993496341021133</v>
+        <v>0.7959867747522211</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>0.3046541359519082</v>
@@ -532,7 +533,7 @@
         <v>0.6499027576921166</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>0.05721201445324109</v>
+        <v>0.05522869601871561</v>
       </c>
     </row>
     <row r="4">
@@ -540,19 +541,19 @@
         <v>1992</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>0.1481055692372539</v>
+        <v>0.1466404541057857</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>0.2020166884846268</v>
+        <v>0.2004876256698491</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>0.214901133021459</v>
+        <v>0.2133523133916952</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>0.431618989708398</v>
+        <v>0.4297954492682905</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>0.4054200029719319</v>
+        <v>0.4036251756221367</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>0.07620457435940065</v>
@@ -561,7 +562,7 @@
         <v>0.08864910610388099</v>
       </c>
       <c r="I4" s="1" t="n">
-        <v>0.03629629134989432</v>
+        <v>0.03498745105596668</v>
       </c>
     </row>
     <row r="5">
@@ -569,19 +570,19 @@
         <v>1993</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.368176146646819</v>
+        <v>0.3667021890339519</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>0.6037332627505605</v>
+        <v>0.6020100080746835</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>0.6710700903446085</v>
+        <v>0.6692767556913606</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>1.072155407752653</v>
+        <v>1.069939157376826</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>1.004604937600635</v>
+        <v>1.002462065840836</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>0.1007787980936903</v>
@@ -590,7 +591,7 @@
         <v>0.1057650929383522</v>
       </c>
       <c r="I5" s="1" t="n">
-        <v>0.03153108027272067</v>
+        <v>0.03041915291796826</v>
       </c>
     </row>
     <row r="6">
@@ -598,19 +599,19 @@
         <v>1994</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.1015297434622657</v>
+        <v>0.09969768183986649</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>0.04792056015303903</v>
+        <v>0.04617673728024485</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>0.06283467750824889</v>
+        <v>0.06106856949746242</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>0.04247962095412716</v>
+        <v>0.04073699260925534</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>0.05681932640850129</v>
+        <v>0.05506015099409622</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>0.01321717705033376</v>
@@ -619,7 +620,7 @@
         <v>0.01503967058350941</v>
       </c>
       <c r="I6" s="1" t="n">
-        <v>0.04487427789095033</v>
+        <v>0.0431516380936352</v>
       </c>
     </row>
     <row r="7">
@@ -627,19 +628,19 @@
         <v>1995</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.3302857400016832</v>
+        <v>0.3277986457430968</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>0.4288554629806118</v>
+        <v>0.4261878552996419</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>0.546950848969449</v>
+        <v>0.5440609242291743</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>0.7149174625561017</v>
+        <v>0.7117267564891014</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>0.7886776785877216</v>
+        <v>0.7853424614183453</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>0.3757621024474107</v>
@@ -648,7 +649,7 @@
         <v>0.4253592895836935</v>
       </c>
       <c r="I7" s="1" t="n">
-        <v>0.05824437772786961</v>
+        <v>0.05626133943275891</v>
       </c>
     </row>
     <row r="8">
@@ -656,19 +657,19 @@
         <v>1996</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.3346892067915641</v>
+        <v>0.332569367718736</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>0.4603915449369489</v>
+        <v>0.4580533940973424</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>0.541535572894934</v>
+        <v>0.539081526908177</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>0.5893011800981554</v>
+        <v>0.586755522589492</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>0.6275200400226697</v>
+        <v>0.62493564615192</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>0.2296096156759775</v>
@@ -677,7 +678,7 @@
         <v>0.425403050865109</v>
       </c>
       <c r="I8" s="1" t="n">
-        <v>0.05341377012322024</v>
+        <v>0.05173015370225587</v>
       </c>
     </row>
     <row r="9">
@@ -685,19 +686,19 @@
         <v>1997</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.3237174243057599</v>
+        <v>0.3212817521008817</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>0.3707185322493673</v>
+        <v>0.3681984028758649</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>0.4100562115587232</v>
+        <v>0.4074647196127275</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>0.5510771085313106</v>
+        <v>0.5482283964742001</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>0.5590831102491318</v>
+        <v>0.5562240346374048</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>0.3336276825136044</v>
@@ -706,7 +707,7 @@
         <v>0.2063285282945373</v>
       </c>
       <c r="I9" s="1" t="n">
-        <v>0.0538351146071645</v>
+        <v>0.05190586990263535</v>
       </c>
     </row>
     <row r="10">
@@ -714,19 +715,19 @@
         <v>1998</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.4525158476209807</v>
+        <v>0.4499582639949358</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>0.5988847000648729</v>
+        <v>0.5960793424986763</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>0.6227433505666427</v>
+        <v>0.619904617802759</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>0.7929734511595365</v>
+        <v>0.7898177193276676</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>0.8461648662710668</v>
+        <v>0.8429224209488639</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>0.2857901787776596</v>
@@ -735,7 +736,7 @@
         <v>0.8530020286022797</v>
       </c>
       <c r="I10" s="1" t="n">
-        <v>0.05068894219075948</v>
+        <v>0.048890086721052</v>
       </c>
     </row>
     <row r="11">
@@ -743,28 +744,28 @@
         <v>1999</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.01973678515583943</v>
+        <v>0.01798402947225086</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>0.08442217417005526</v>
+        <v>0.08255573466084387</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>0.107884544121172</v>
+        <v>0.1059781664094566</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>0.1160523527959887</v>
+        <v>0.1141278588244565</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>0.1590362407450898</v>
+        <v>0.1570375058791929</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>0.210411913701116</v>
       </c>
       <c r="H11" s="1" t="n">
-        <v>0.986838583091173</v>
+        <v>1.019504251066171</v>
       </c>
       <c r="I11" s="1" t="n">
-        <v>0.04924135334993696</v>
+        <v>0.04743737511732715</v>
       </c>
     </row>
     <row r="12">
@@ -772,28 +773,28 @@
         <v>2000</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.3473292428266599</v>
+        <v>0.3445632671123116</v>
       </c>
       <c r="C12" s="1" t="n">
-        <v>0.3976136369217216</v>
+        <v>0.3947481444613861</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>0.4644559646320983</v>
+        <v>0.4614528239716063</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>0.5710716987913491</v>
+        <v>0.5678583155376673</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>0.6800090220523796</v>
+        <v>0.676574483211495</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>-0.09104086276837975</v>
       </c>
       <c r="H12" s="1" t="n">
-        <v>-0.3611491036928773</v>
+        <v>-0.3684446158534768</v>
       </c>
       <c r="I12" s="1" t="n">
-        <v>0.06183297271042232</v>
+        <v>0.05964987851852044</v>
       </c>
     </row>
     <row r="13">
@@ -801,28 +802,28 @@
         <v>2001</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.1303871211279843</v>
+        <v>0.129368444467912</v>
       </c>
       <c r="C13" s="1" t="n">
-        <v>0.1791239794652892</v>
+        <v>0.1780640351720322</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>0.2652017172245402</v>
+        <v>0.2640673761179855</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>0.3995704401484719</v>
+        <v>0.3983061702156943</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>0.4720759837682531</v>
+        <v>0.470748213060403</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>-0.1188601098308978</v>
       </c>
       <c r="H13" s="1" t="n">
-        <v>-0.3334472990133833</v>
+        <v>-0.3265362770636708</v>
       </c>
       <c r="I13" s="1" t="n">
-        <v>0.03582948491767279</v>
+        <v>0.03490918866214732</v>
       </c>
     </row>
     <row r="14">
@@ -830,28 +831,28 @@
         <v>2002</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.2911271181683668</v>
+        <v>0.2903842755344743</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>0.3048596895651177</v>
+        <v>0.3041111360237019</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>0.3518340448450112</v>
+        <v>0.3510615112130158</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>0.3562767779749796</v>
+        <v>0.3555046558241937</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>0.3828287012946354</v>
+        <v>0.3820439540717611</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>-0.221003347786878</v>
       </c>
       <c r="H14" s="1" t="n">
-        <v>-0.3736840819716171</v>
+        <v>-0.3758156050854439</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>0.01673679128194716</v>
+        <v>0.01615418449548889</v>
       </c>
     </row>
     <row r="15">
@@ -859,19 +860,19 @@
         <v>2003</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.4494033328020428</v>
+        <v>0.4488731708681346</v>
       </c>
       <c r="C15" s="1" t="n">
-        <v>0.332681997545742</v>
+        <v>0.3321926367712649</v>
       </c>
       <c r="D15" s="1" t="n">
-        <v>0.3857980281317939</v>
+        <v>0.3852890546801468</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>0.4041217779443818</v>
+        <v>0.4036077369390723</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>0.4514365862293153</v>
+        <v>0.4509053907640321</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>0.2868424808512648</v>
@@ -880,7 +881,7 @@
         <v>0.4966900007799731</v>
       </c>
       <c r="I15" s="1" t="n">
-        <v>0.0105025730043975</v>
+        <v>0.01013071119385645</v>
       </c>
     </row>
     <row r="16">
@@ -888,19 +889,19 @@
         <v>2004</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.1835898210961016</v>
+        <v>0.1828774680293888</v>
       </c>
       <c r="C16" s="1" t="n">
-        <v>0.1820792095113621</v>
+        <v>0.1813631399632034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>0.2315121494621692</v>
+        <v>0.2307663441981109</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>0.2619481122459815</v>
+        <v>0.2611879546709002</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>0.2857325829295565</v>
+        <v>0.2849572039110768</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>0.1088210285038285</v>
@@ -909,7 +910,7 @@
         <v>0.1053855549222371</v>
       </c>
       <c r="I16" s="1" t="n">
-        <v>0.0144079319202326</v>
+        <v>0.01379041498544464</v>
       </c>
     </row>
     <row r="17">
@@ -917,19 +918,19 @@
         <v>2005</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>-0.05692081841368746</v>
+        <v>-0.05806869473622134</v>
       </c>
       <c r="C17" s="1" t="n">
-        <v>0.06045208096850119</v>
+        <v>0.05915740944400527</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>0.07232941783422242</v>
+        <v>0.0710217982484902</v>
       </c>
       <c r="E17" s="1" t="n">
-        <v>0.07703172681031933</v>
+        <v>0.07571972039551644</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>0.1063907689657486</v>
+        <v>0.1050463993569715</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>0.04911783501431088</v>
@@ -938,7 +939,7 @@
         <v>0.01565202530489662</v>
       </c>
       <c r="I17" s="1" t="n">
-        <v>0.0330526457999103</v>
+        <v>0.0317920801504874</v>
       </c>
     </row>
     <row r="18">
@@ -946,19 +947,19 @@
         <v>2006</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.07634111694842116</v>
+        <v>0.07450247911618568</v>
       </c>
       <c r="C18" s="1" t="n">
-        <v>0.1449555235191362</v>
+        <v>0.1430019975132018</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>0.1558406284277414</v>
+        <v>0.1538648771786606</v>
       </c>
       <c r="E18" s="1" t="n">
-        <v>0.2336224635175976</v>
+        <v>0.2315102337047577</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>0.2331838693771</v>
+        <v>0.2310698958937052</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>0.157944638071126</v>
@@ -967,7 +968,7 @@
         <v>0.07144328431386748</v>
       </c>
       <c r="I18" s="1" t="n">
-        <v>0.04996968189242024</v>
+        <v>0.04818327970600866</v>
       </c>
     </row>
     <row r="19">
@@ -975,19 +976,19 @@
         <v>2007</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.1531189288528041</v>
+        <v>0.1516050745567652</v>
       </c>
       <c r="C19" s="1" t="n">
-        <v>0.1369601273053236</v>
+        <v>0.1354699759382934</v>
       </c>
       <c r="D19" s="1" t="n">
-        <v>0.202026823764256</v>
+        <v>0.2004599534737739</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>0.2470448662631566</v>
+        <v>0.2454130384438256</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>0.2791577664019045</v>
+        <v>0.2774901977306448</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>0.05493726356621176</v>
@@ -996,7 +997,7 @@
         <v>0.1902799476875014</v>
       </c>
       <c r="I19" s="1" t="n">
-        <v>0.04613036596297992</v>
+        <v>0.04475014514205888</v>
       </c>
     </row>
     <row r="20">
@@ -1004,19 +1005,19 @@
         <v>2008</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.9960870638464276</v>
+        <v>0.9951523539798106</v>
       </c>
       <c r="C20" s="1" t="n">
-        <v>1.06365544316022</v>
+        <v>1.062693446516214</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>0.950813749363894</v>
+        <v>0.9499047441531956</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>0.8712749305519383</v>
+        <v>0.8704063370082791</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>0.8083989549664168</v>
+        <v>0.8075598979966541</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>-0.3699761081938914</v>
@@ -1025,7 +1026,7 @@
         <v>-0.4172723405513733</v>
       </c>
       <c r="I20" s="1" t="n">
-        <v>0.01434585314311354</v>
+        <v>0.01387279554442689</v>
       </c>
     </row>
     <row r="21">
@@ -1033,19 +1034,19 @@
         <v>2009</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.2280629125576425</v>
+        <v>-0.228120933701747</v>
       </c>
       <c r="C21" s="1" t="n">
-        <v>-0.1386620011560769</v>
+        <v>-0.1387263635251382</v>
       </c>
       <c r="D21" s="1" t="n">
-        <v>-0.08808595614599746</v>
+        <v>-0.08815404193126686</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>-0.03453575392786423</v>
+        <v>-0.03460709262026862</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>-0.01504989946397595</v>
+        <v>-0.01512269953382983</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>0.264642321298298</v>
@@ -1054,7 +1055,7 @@
         <v>0.5468432209179339</v>
       </c>
       <c r="I21" s="1" t="n">
-        <v>0.001551196248863462</v>
+        <v>0.001476973522390512</v>
       </c>
     </row>
     <row r="22">
@@ -1062,19 +1063,19 @@
         <v>2010</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.2011378388834419</v>
+        <v>0.2010613603644784</v>
       </c>
       <c r="C22" s="1" t="n">
-        <v>0.2401055525335773</v>
+        <v>0.2400270847746733</v>
       </c>
       <c r="D22" s="1" t="n">
-        <v>0.2662169584218217</v>
+        <v>0.2661366676282273</v>
       </c>
       <c r="E22" s="1" t="n">
-        <v>0.3996123692365299</v>
+        <v>0.3995236572271494</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>0.3938667192488003</v>
+        <v>0.3937783905274417</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>0.15063401360544</v>
@@ -1083,7 +1084,7 @@
         <v>0.2014364886282187</v>
       </c>
       <c r="I22" s="1" t="n">
-        <v>0.001429190828477145</v>
+        <v>0.001366681595040609</v>
       </c>
     </row>
     <row r="23">
@@ -1091,19 +1092,19 @@
         <v>2011</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.1786244994459034</v>
+        <v>-0.1786404996437959</v>
       </c>
       <c r="C23" s="1" t="n">
-        <v>-0.04065362649377169</v>
+        <v>-0.04067232355934247</v>
       </c>
       <c r="D23" s="1" t="n">
-        <v>-0.03833807833410963</v>
+        <v>-0.03835681347270736</v>
       </c>
       <c r="E23" s="1" t="n">
-        <v>-0.004465953383957166</v>
+        <v>-0.004485333470451103</v>
       </c>
       <c r="F23" s="1" t="n">
-        <v>-0.04233039358068158</v>
+        <v>-0.04234901031661931</v>
       </c>
       <c r="G23" s="1" t="n">
         <v>0.02111820043608126</v>
@@ -1112,7 +1113,7 @@
         <v>0.03475807772937101</v>
       </c>
       <c r="I23" s="1" t="n">
-        <v>0.0005422094031992675</v>
+        <v>0.0005228751307688739</v>
       </c>
     </row>
     <row r="24">
@@ -1120,19 +1121,19 @@
         <v>2012</v>
       </c>
       <c r="B24" s="1" t="n">
-        <v>-0.1411007929969329</v>
+        <v>-0.1411359140519999</v>
       </c>
       <c r="C24" s="1" t="n">
-        <v>-0.1167338140742247</v>
+        <v>-0.1167700130276567</v>
       </c>
       <c r="D24" s="1" t="n">
-        <v>-0.1424573966108182</v>
+        <v>-0.1424924965621783</v>
       </c>
       <c r="E24" s="1" t="n">
-        <v>-0.1226292691814905</v>
+        <v>-0.1226649689118057</v>
       </c>
       <c r="F24" s="1" t="n">
-        <v>-0.1111851918311163</v>
+        <v>-0.1112213038836686</v>
       </c>
       <c r="G24" s="1" t="n">
         <v>0.1600322380427452</v>
@@ -1141,7 +1142,7 @@
         <v>0.1811253955977239</v>
       </c>
       <c r="I24" s="1" t="n">
-        <v>0.0009055668352333512</v>
+        <v>0.0008644810626574628</v>
       </c>
     </row>
     <row r="25">
@@ -1149,19 +1150,19 @@
         <v>2013</v>
       </c>
       <c r="B25" s="1" t="n">
-        <v>0.0328753810644753</v>
+        <v>0.03284853277736088</v>
       </c>
       <c r="C25" s="1" t="n">
-        <v>0.03692192361804514</v>
+        <v>0.03689491476386597</v>
       </c>
       <c r="D25" s="1" t="n">
-        <v>0.03548941813520301</v>
+        <v>0.03546240578303461</v>
       </c>
       <c r="E25" s="1" t="n">
-        <v>0.101548842183768</v>
+        <v>0.1015201480415384</v>
       </c>
       <c r="F25" s="1" t="n">
-        <v>0.1010250194843882</v>
+        <v>0.1009962598936542</v>
       </c>
       <c r="G25" s="1" t="n">
         <v>0.3238847806296004</v>
@@ -1170,7 +1171,7 @@
         <v>0.3663422322212719</v>
       </c>
       <c r="I25" s="1" t="n">
-        <v>0.0005942232934741387</v>
+        <v>0.0005681055567328119</v>
       </c>
     </row>
     <row r="26">
@@ -1178,19 +1179,19 @@
         <v>2014</v>
       </c>
       <c r="B26" s="1" t="n">
-        <v>0.3936436453978223</v>
+        <v>0.393621748726267</v>
       </c>
       <c r="C26" s="1" t="n">
-        <v>0.5347330811945783</v>
+        <v>0.5347089734709158</v>
       </c>
       <c r="D26" s="1" t="n">
-        <v>0.6422415097334451</v>
+        <v>0.6422157733994438</v>
       </c>
       <c r="E26" s="1" t="n">
-        <v>0.7907126067341159</v>
+        <v>0.7906846579797124</v>
       </c>
       <c r="F26" s="1" t="n">
-        <v>0.8232497236405498</v>
+        <v>0.8232213307676823</v>
       </c>
       <c r="G26" s="1" t="n">
         <v>0.1368836315708499</v>
@@ -1199,7 +1200,7 @@
         <v>0.1918141645796192</v>
       </c>
       <c r="I26" s="1" t="n">
-        <v>0.0003369612625909735</v>
+        <v>0.0003211471355331064</v>
       </c>
     </row>
     <row r="27">
@@ -1207,19 +1208,19 @@
         <v>2015</v>
       </c>
       <c r="B27" s="1" t="n">
-        <v>-0.02199043351228158</v>
+        <v>-0.02203207450625788</v>
       </c>
       <c r="C27" s="1" t="n">
-        <v>0.004133177421054013</v>
+        <v>0.004090367647606064</v>
       </c>
       <c r="D27" s="1" t="n">
-        <v>0.05480718223649195</v>
+        <v>0.0547621457500802</v>
       </c>
       <c r="E27" s="1" t="n">
-        <v>0.07007871813755351</v>
+        <v>0.07003313436869152</v>
       </c>
       <c r="F27" s="1" t="n">
-        <v>0.1021442800989631</v>
+        <v>0.1020973569291126</v>
       </c>
       <c r="G27" s="1" t="n">
         <v>0.01383759921898431</v>
@@ -1228,7 +1229,7 @@
         <v>0.09435423949203803</v>
       </c>
       <c r="I27" s="1" t="n">
-        <v>0.000544591224157509</v>
+        <v>0.0005025904769846434</v>
       </c>
     </row>
     <row r="28">
@@ -1236,19 +1237,19 @@
         <v>2016</v>
       </c>
       <c r="B28" s="1" t="n">
-        <v>-0.1726879389827551</v>
+        <v>-0.1728150195624474</v>
       </c>
       <c r="C28" s="1" t="n">
-        <v>-0.1072347408268292</v>
+        <v>-0.107371685095662</v>
       </c>
       <c r="D28" s="1" t="n">
-        <v>-0.1002217263101497</v>
+        <v>-0.1003597733758548</v>
       </c>
       <c r="E28" s="1" t="n">
-        <v>-0.1512454732882036</v>
+        <v>-0.1513751609459206</v>
       </c>
       <c r="F28" s="1" t="n">
-        <v>-0.1810728421086254</v>
+        <v>-0.1811981234041404</v>
       </c>
       <c r="G28" s="1" t="n">
         <v>0.1195991207871063</v>
@@ -1257,7 +1258,7 @@
         <v>0.07098286188239489</v>
       </c>
       <c r="I28" s="1" t="n">
-        <v>0.003287114685658787</v>
+        <v>0.003133640586880038</v>
       </c>
     </row>
     <row r="29">
@@ -1265,19 +1266,19 @@
         <v>2017</v>
       </c>
       <c r="B29" s="1" t="n">
-        <v>-0.1243188283203407</v>
+        <v>-0.1246598353409596</v>
       </c>
       <c r="C29" s="1" t="n">
-        <v>-0.07921420012731761</v>
+        <v>-0.07957347839765949</v>
       </c>
       <c r="D29" s="1" t="n">
-        <v>-0.08926024192178872</v>
+        <v>-0.08961512855142884</v>
       </c>
       <c r="E29" s="1" t="n">
-        <v>-0.1441783707061793</v>
+        <v>-0.1445118848970263</v>
       </c>
       <c r="F29" s="1" t="n">
-        <v>-0.1350681202666238</v>
+        <v>-0.1354045877411718</v>
       </c>
       <c r="G29" s="1" t="n">
         <v>0.2183160148270713</v>
@@ -1286,7 +1287,7 @@
         <v>0.326636469242753</v>
       </c>
       <c r="I29" s="1" t="n">
-        <v>0.009667671520190435</v>
+        <v>0.009272910567206916</v>
       </c>
     </row>
     <row r="30">
@@ -1294,19 +1295,19 @@
         <v>2018</v>
       </c>
       <c r="B30" s="1" t="n">
-        <v>-0.07915772307375646</v>
+        <v>-0.07977264727082733</v>
       </c>
       <c r="C30" s="1" t="n">
-        <v>-0.05437841152766099</v>
+        <v>-0.05501063281388485</v>
       </c>
       <c r="D30" s="1" t="n">
-        <v>-0.04012256160095085</v>
+        <v>-0.04076503888614413</v>
       </c>
       <c r="E30" s="1" t="n">
-        <v>-0.06940329240881338</v>
+        <v>-0.07002698926028472</v>
       </c>
       <c r="F30" s="1" t="n">
-        <v>0.02346847607195457</v>
+        <v>0.02278256815373725</v>
       </c>
       <c r="G30" s="1" t="n">
         <v>-0.0438424174525569</v>
@@ -1315,7 +1316,7 @@
         <v>-0.001262566267758447</v>
       </c>
       <c r="I30" s="1" t="n">
-        <v>0.02027017051082791</v>
+        <v>0.01959148166144886</v>
       </c>
     </row>
     <row r="31">
@@ -1323,19 +1324,19 @@
         <v>2019</v>
       </c>
       <c r="B31" s="1" t="n">
-        <v>-0.05637958853307923</v>
+        <v>-0.05708282454750491</v>
       </c>
       <c r="C31" s="1" t="n">
-        <v>0.04115978304755186</v>
+        <v>0.04038548564085676</v>
       </c>
       <c r="D31" s="1" t="n">
-        <v>0.1066285399851143</v>
+        <v>0.1058063003112779</v>
       </c>
       <c r="E31" s="1" t="n">
-        <v>0.1672932160942509</v>
+        <v>0.1664272465871914</v>
       </c>
       <c r="F31" s="1" t="n">
-        <v>0.2279302661700926</v>
+        <v>0.2270204969116345</v>
       </c>
       <c r="G31" s="1" t="n">
         <v>0.3148637098683436</v>
@@ -1344,7 +1345,7 @@
         <v>0.389613478961214</v>
       </c>
       <c r="I31" s="1" t="n">
-        <v>0.02157173616791308</v>
+        <v>0.02081335978505661</v>
       </c>
     </row>
     <row r="32">
@@ -1352,19 +1353,19 @@
         <v>2020</v>
       </c>
       <c r="B32" s="1" t="n">
-        <v>0.0797493034568888</v>
+        <v>0.07963434487647802</v>
       </c>
       <c r="C32" s="1" t="n">
-        <v>0.3849911090164657</v>
+        <v>0.3848448605666992</v>
       </c>
       <c r="D32" s="1" t="n">
-        <v>0.5333700598988602</v>
+        <v>0.5332088471049172</v>
       </c>
       <c r="E32" s="1" t="n">
-        <v>0.8012264313431927</v>
+        <v>0.8010377947631655</v>
       </c>
       <c r="F32" s="1" t="n">
-        <v>0.8641202245224049</v>
+        <v>0.8639269463977821</v>
       </c>
       <c r="G32" s="1" t="n">
         <v>0.1839882689892662</v>
@@ -1373,7 +1374,7 @@
         <v>0.4840651869821666</v>
       </c>
       <c r="I32" s="1" t="n">
-        <v>0.003762532532923579</v>
+        <v>0.003658352876944715</v>
       </c>
     </row>
     <row r="33">
@@ -1381,19 +1382,19 @@
         <v>2021</v>
       </c>
       <c r="B33" s="1" t="n">
-        <v>0.326883520536462</v>
+        <v>0.3268610442359634</v>
       </c>
       <c r="C33" s="1" t="n">
-        <v>0.3765243948322559</v>
+        <v>0.3765011220791668</v>
       </c>
       <c r="D33" s="1" t="n">
-        <v>0.3640202484429789</v>
+        <v>0.3639971497507624</v>
       </c>
       <c r="E33" s="1" t="n">
-        <v>0.4354581174664158</v>
+        <v>0.435433732449338</v>
       </c>
       <c r="F33" s="1" t="n">
-        <v>0.3642337537082561</v>
+        <v>0.3642105633675246</v>
       </c>
       <c r="G33" s="1" t="n">
         <v>0.2870536836204058</v>
@@ -1402,7 +1403,7 @@
         <v>0.2741959404012131</v>
       </c>
       <c r="I33" s="1" t="n">
-        <v>0.0004711421957845907</v>
+        <v>0.0004543491391522103</v>
       </c>
     </row>
     <row r="34">
@@ -1410,19 +1411,19 @@
         <v>2022</v>
       </c>
       <c r="B34" s="1" t="n">
-        <v>0.2586845358225127</v>
+        <v>0.257356651701095</v>
       </c>
       <c r="C34" s="1" t="n">
-        <v>0.2871688057845152</v>
+        <v>0.2858102521909065</v>
       </c>
       <c r="D34" s="1" t="n">
-        <v>0.2376410377544822</v>
+        <v>0.2363372797408965</v>
       </c>
       <c r="E34" s="1" t="n">
-        <v>0.4523555839460185</v>
+        <v>0.4508257612265307</v>
       </c>
       <c r="F34" s="1" t="n">
-        <v>0.3534491309651531</v>
+        <v>0.3520254522329087</v>
       </c>
       <c r="G34" s="1" t="n">
         <v>-0.181108874803489</v>
@@ -1431,7 +1432,7 @@
         <v>-0.3257705080852904</v>
       </c>
       <c r="I34" s="1" t="n">
-        <v>0.02118912856690836</v>
+        <v>0.02011425446538673</v>
       </c>
     </row>
     <row r="35">
@@ -1439,19 +1440,19 @@
         <v>2023</v>
       </c>
       <c r="B35" s="1" t="n">
-        <v>-0.0854973549640512</v>
+        <v>-0.08715706062124318</v>
       </c>
       <c r="C35" s="1" t="n">
-        <v>-0.03890059286396619</v>
+        <v>-0.0406513510796106</v>
       </c>
       <c r="D35" s="1" t="n">
-        <v>-0.0325748862834665</v>
+        <v>-0.03433488072223079</v>
       </c>
       <c r="E35" s="1" t="n">
-        <v>-0.1229852567809153</v>
+        <v>-0.1245759175595101</v>
       </c>
       <c r="F35" s="1" t="n">
-        <v>-0.1045771195586179</v>
+        <v>-0.1061990921304856</v>
       </c>
       <c r="G35" s="1" t="n">
         <v>0.2628729203401294</v>
@@ -1460,7 +1461,7 @@
         <v>0.5485583636391509</v>
       </c>
       <c r="I35" s="1" t="n">
-        <v>0.05368206288261623</v>
+        <v>0.05174363544728533</v>
       </c>
     </row>
     <row r="36">
@@ -1468,19 +1469,19 @@
         <v>2024</v>
       </c>
       <c r="B36" s="1" t="n">
-        <v>-0.06963208689979627</v>
+        <v>-0.07104924471828455</v>
       </c>
       <c r="C36" s="1" t="n">
-        <v>-0.06206853139968049</v>
+        <v>-0.06350245639929819</v>
       </c>
       <c r="D36" s="1" t="n">
-        <v>-0.07023131726421927</v>
+        <v>-0.07165008715876309</v>
       </c>
       <c r="E36" s="1" t="n">
-        <v>-0.1322492844918777</v>
+        <v>-0.1335710401308361</v>
       </c>
       <c r="F36" s="1" t="n">
-        <v>-0.1425202457452681</v>
+        <v>-0.1438248563702592</v>
       </c>
       <c r="G36" s="1" t="n">
         <v>0.2501984933867818</v>
@@ -1489,7 +1490,7 @@
         <v>0.2557819219564408</v>
       </c>
       <c r="I36" s="1" t="n">
-        <v>0.05300925641922638</v>
+        <v>0.05139370285685563</v>
       </c>
     </row>
     <row r="37">
@@ -1497,19 +1498,19 @@
         <v>2025</v>
       </c>
       <c r="B37" s="1" t="n">
-        <v>-0.05641232122598294</v>
+        <v>-0.05778884377167803</v>
       </c>
       <c r="C37" s="1" t="n">
-        <v>0.02215515094975329</v>
+        <v>0.02066426274250843</v>
       </c>
       <c r="D37" s="1" t="n">
-        <v>0.002151767440493391</v>
+        <v>0.0006880915767792928</v>
       </c>
       <c r="E37" s="1" t="n">
-        <v>0.0327622827769658</v>
+        <v>0.03124535553289443</v>
       </c>
       <c r="F37" s="1" t="n">
-        <v>0.01990096612110248</v>
+        <v>0.01840297009220304</v>
       </c>
       <c r="G37" s="1" t="n">
         <v>0.1788054337892473</v>
@@ -1518,7 +1519,7 @@
         <v>0.2077254184059141</v>
       </c>
       <c r="I37" s="1" t="n">
-        <v>0.04299604947156643</v>
+        <v>0.04149269687022561</v>
       </c>
     </row>
     <row r="38">
@@ -1528,19 +1529,19 @@
         </is>
       </c>
       <c r="B38" s="1" t="n">
-        <v>0.0508238643317005</v>
+        <v>0.05001764264473074</v>
       </c>
       <c r="C38" s="1" t="n">
-        <v>0.05134765346649517</v>
+        <v>0.05054862241649349</v>
       </c>
       <c r="D38" s="1" t="n">
-        <v>0.03178958813767707</v>
+        <v>0.03100897033523875</v>
       </c>
       <c r="E38" s="1" t="n">
-        <v>-0.001457158757461219</v>
+        <v>-0.002217512248365971</v>
       </c>
       <c r="F38" s="1" t="n">
-        <v>-0.02126021450804449</v>
+        <v>-0.02200385432967089</v>
       </c>
       <c r="G38" s="1" t="n">
         <v>0.113603363884234</v>
@@ -1549,7 +1550,7 @@
         <v>0.1838049736616416</v>
       </c>
       <c r="I38" s="1" t="n">
-        <v>0.01984370409772063</v>
+        <v>0.01907379014574362</v>
       </c>
     </row>
   </sheetData>
@@ -1563,7 +1564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1625,29 +1626,29 @@
           <t>CAGR (rendement total)</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>0.1313877159362955</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>0.1945314254699106</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>0.2239917043732078</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>0.2820747786675974</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>0.2972981334590807</v>
-      </c>
-      <c r="G2" s="2" t="n">
+      <c r="B2" s="1" t="n">
+        <v>0.1302869952734138</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>0.1933687562137414</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>0.2228013084703142</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>0.2808263551231407</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>0.2960365429272604</v>
+      </c>
+      <c r="G2" s="1" t="n">
         <v>0.1096359552701101</v>
       </c>
-      <c r="H2" s="2" t="n">
-        <v>0.1477924094523611</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>0.02862082239780439</v>
+      <c r="H2" s="1" t="n">
+        <v>0.1481610484260478</v>
+      </c>
+      <c r="I2" s="1" t="n">
+        <v>0.02762141779089999</v>
       </c>
     </row>
     <row r="3">
@@ -1656,26 +1657,26 @@
           <t>CAGR au même risque que le S&amp;P 500</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>0.1090607259481344</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>0.1963261977632853</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>0.2194102809991425</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>0.2419590412240515</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>0.2518656569720723</v>
-      </c>
-      <c r="G3" s="2" t="n">
+      <c r="B3" s="1" t="n">
+        <v>0.1079780162416877</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>0.1951515965993202</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0.2182125463322897</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>0.2407366417047963</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>0.2506342468450735</v>
+      </c>
+      <c r="G3" s="1" t="n">
         <v>0.1096359552701101</v>
       </c>
-      <c r="H3" s="2" t="n">
-        <v>0.1176716074512338</v>
+      <c r="H3" s="1" t="n">
+        <v>0.1173469656165522</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -1685,29 +1686,29 @@
           <t>Volatilité annualisée (écart-type quotidien)</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>0.2459136743571607</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>0.1763084449775143</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>0.1826534079141405</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>0.2118084650496137</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>0.2142411114145703</v>
-      </c>
-      <c r="G4" s="2" t="n">
+      <c r="B4" s="1" t="n">
+        <v>0.2459233373921978</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>0.1763250221812348</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>0.1826655064854853</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>0.2118253500359789</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>0.2142519093467997</v>
+      </c>
+      <c r="G4" s="1" t="n">
         <v>0.1782698674551475</v>
       </c>
-      <c r="H4" s="2" t="n">
-        <v>0.2577533726979754</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>0.001393232042974603</v>
+      <c r="H4" s="1" t="n">
+        <v>0.2587351798928421</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>0.001818081392500849</v>
       </c>
     </row>
     <row r="5">
@@ -1716,388 +1717,442 @@
           <t>Écart-type des performances annuelles</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>0.260632508100315</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>0.2721565839697694</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>0.2854671155148205</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>0.3551356523025335</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>0.3639635541974695</v>
-      </c>
-      <c r="G5" s="2" t="n">
+      <c r="B5" s="1" t="n">
+        <v>0.2601594648097524</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>0.271665380288315</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0.284911239997391</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>0.3544755330590767</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>0.3632185668971095</v>
+      </c>
+      <c r="G5" s="1" t="n">
         <v>0.1732061170079772</v>
       </c>
-      <c r="H5" s="2" t="n">
-        <v>0.3266895064322894</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>0.02337710333635718</v>
+      <c r="H5" s="1" t="n">
+        <v>0.3291433702250893</v>
+      </c>
+      <c r="I5" s="1" t="n">
+        <v>0.02257345678083112</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sharpe</t>
+          <t>Exposition moyenne (notionnel / capital)</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.504123301080828</v>
+        <v>5.255551551898108</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.9209189642025855</v>
+        <v>5.595593451885319</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1.026184098168938</v>
+        <v>6.773347111599876</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1.126977431429837</v>
+        <v>7.778758350633463</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1.170743636605178</v>
+        <v>8.783663406381326</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.5066419367211662</v>
+        <v>1</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.5461432844593563</v>
+        <v>1</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sortino</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>0.7062859067510308</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>1.309338369697399</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>1.464741550233657</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>1.630809212784845</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>1.703522897641643</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>0.7168223016023005</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>0.7844552214122501</v>
-      </c>
+          <t>Coûts par an (transactions + roulement)</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>0.01293996377788859</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>0.01405248005523779</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>0.01701685995733537</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>0.0214650795201738</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>0.02464228138215597</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Calmar (CAGR / pire baisse)</t>
+          <t>Sharpe</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.1967625303245683</v>
+        <v>0.504123301080828</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.4843678217805872</v>
+        <v>0.9209189642025855</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.5422036722295268</v>
+        <v>1.026184098168938</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.5853201196617522</v>
+        <v>1.126977431429837</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.6252122669351092</v>
+        <v>1.170743636605178</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.198435248503774</v>
+        <v>0.5120073849991348</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0.1781406866690624</v>
+        <v>0.5498640582639125</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pire baisse (max drawdown)</t>
+          <t>Sortino</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>-0.6677476434134376</v>
+        <v>0.7062859067510308</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.4016192173022407</v>
+        <v>1.309338369697399</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>-0.4131135878371314</v>
+        <v>1.464741550233657</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-0.4819153984158349</v>
+        <v>1.630809212784845</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-0.4755155155807864</v>
+        <v>1.703522897641643</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>-0.5525024213025587</v>
+        <v>0.7246495686932037</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>-0.8296387098076012</v>
+        <v>0.7925777239820938</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Meilleure année</t>
+          <t>Calmar (CAGR / pire baisse)</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.9960870638464276</v>
+        <v>0.194888501931789</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>1.06365544316022</v>
+        <v>0.4806382436388979</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.950813749363894</v>
+        <v>0.5384519349589575</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>1.072155407752653</v>
+        <v>0.5799043228477244</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>1.113519887330518</v>
+        <v>0.6194668410427379</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.3757621024474107</v>
+        <v>0.198435248503774</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0.986838583091173</v>
-      </c>
-      <c r="I10" s="2" t="n">
-        <v>0.08066065701536451</v>
-      </c>
+        <v>0.1787286266115603</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Pire année</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>-0.2280629125576425</v>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>-0.1386620011560769</v>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>-0.1424573966108182</v>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>-0.1512454732882036</v>
-      </c>
-      <c r="F11" s="2" t="n">
-        <v>-0.1810728421086254</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>-0.3699761081938914</v>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>-0.4172723405513733</v>
-      </c>
-      <c r="I11" s="2" t="n">
-        <v>0.0003369612625909735</v>
-      </c>
+          <t>Pire baisse (max drawdown)</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>-0.6685206873775154</v>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>-0.4023166253890915</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>-0.4137812384076526</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>-0.4842632552626827</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>-0.4778892481620924</v>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>-0.5525024213025587</v>
+      </c>
+      <c r="H11" s="1" t="n">
+        <v>-0.8289721195477741</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Années positives</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>0.8055555555555556</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>0.8055555555555556</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>0.8055555555555556</v>
-      </c>
-      <c r="I12" s="2" t="n">
-        <v>1</v>
+          <t>Meilleure année</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>0.9951523539798106</v>
+      </c>
+      <c r="C12" s="1" t="n">
+        <v>1.062693446516214</v>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>0.9499047441531956</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>1.069939157376826</v>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>1.107785016528875</v>
+      </c>
+      <c r="G12" s="1" t="n">
+        <v>0.3757621024474107</v>
+      </c>
+      <c r="H12" s="1" t="n">
+        <v>1.019504251066171</v>
+      </c>
+      <c r="I12" s="1" t="n">
+        <v>0.07774330018656528</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Pire mois</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>-0.2286893268739112</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>-0.1074379876370939</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>-0.1386073546428309</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>-0.1427720359974595</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>-0.1318766414445331</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>-0.1679506188757092</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>-0.2620526558891454</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>9.920681374397944e-06</v>
+          <t>Pire année</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>-0.228120933701747</v>
+      </c>
+      <c r="C13" s="1" t="n">
+        <v>-0.1387263635251382</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>-0.1424924965621783</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>-0.1513751609459206</v>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>-0.1811981234041404</v>
+      </c>
+      <c r="G13" s="1" t="n">
+        <v>-0.3699761081938914</v>
+      </c>
+      <c r="H13" s="1" t="n">
+        <v>-0.4172723405513733</v>
+      </c>
+      <c r="I13" s="1" t="n">
+        <v>0.0003211471355331064</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mois positifs</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>0.5580865603644647</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>0.6082004555808656</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>0.5945330296127562</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>0.6036446469248291</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>0.5945330296127562</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>0.6605922551252847</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>0.6059225512528473</v>
-      </c>
-      <c r="I14" s="2" t="n">
+          <t>Années positives</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="C14" s="1" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="F14" s="1" t="n">
+        <v>0.8055555555555556</v>
+      </c>
+      <c r="G14" s="1" t="n">
+        <v>0.8055555555555556</v>
+      </c>
+      <c r="H14" s="1" t="n">
+        <v>0.8055555555555556</v>
+      </c>
+      <c r="I14" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Skew mensuel</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>1.105771241789423</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>0.7278432177471821</v>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>0.5895201062878646</v>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>0.6234652080603125</v>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>0.5829434614726743</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>-0.5253980973034242</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>-0.26874742677639</v>
-      </c>
-      <c r="I15" t="inlineStr"/>
+          <t>Pire mois</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>-0.2286919819128725</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>-0.1075625574043143</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>-0.1386515614545532</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>-0.1430218737499565</v>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>-0.1319205626259774</v>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>-0.1679506188757092</v>
+      </c>
+      <c r="H15" s="1" t="n">
+        <v>-0.2640493636714231</v>
+      </c>
+      <c r="I15" s="1" t="n">
+        <v>8.219207205728551e-06</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Corrélation S&amp;P 500 (mensuelle)</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>-0.3054110632900202</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>-0.2214204997288789</v>
-      </c>
-      <c r="D16" s="2" t="n">
-        <v>-0.1529240139803486</v>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>-0.1357941083426057</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>-0.09877601815219852</v>
-      </c>
-      <c r="G16" s="2" t="n">
+          <t>Mois positifs</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>0.5558086560364465</v>
+      </c>
+      <c r="C16" s="1" t="n">
+        <v>0.6082004555808656</v>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>0.5945330296127562</v>
+      </c>
+      <c r="E16" s="1" t="n">
+        <v>0.6036446469248291</v>
+      </c>
+      <c r="F16" s="1" t="n">
+        <v>0.592255125284738</v>
+      </c>
+      <c r="G16" s="1" t="n">
+        <v>0.6605922551252847</v>
+      </c>
+      <c r="H16" s="1" t="n">
+        <v>0.6059225512528473</v>
+      </c>
+      <c r="I16" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H16" s="2" t="n">
-        <v>0.8368658497092523</v>
-      </c>
-      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Skew mensuel</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>1.106328521216587</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>0.7282803818480869</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>0.5901193147340306</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>0.6235844659986115</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0.5830987956540321</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>-0.5253980973034242</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>-0.2612078332961718</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Corrélation S&amp;P 500 (mensuelle)</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>-0.3053556819433638</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>-0.2214006320663197</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>-0.1529236705548208</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>-0.1357812095606725</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>-0.09877120087794164</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0.9999999999999999</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0.8361536794853948</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>Corrélation Nasdaq-100 (mensuelle)</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
-        <v>-0.2715228483469909</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>-0.1980123937149502</v>
-      </c>
-      <c r="D17" s="2" t="n">
-        <v>-0.1484456694063989</v>
-      </c>
-      <c r="E17" s="2" t="n">
-        <v>-0.1317351185172729</v>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>-0.1041020202992237</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>0.8368658497092523</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I17" t="inlineStr"/>
+      <c r="B19" s="2" t="n">
+        <v>-0.2715858707605233</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>-0.1980596580337521</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>-0.148646658167275</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>-0.131649794131855</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>-0.1041825689321195</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0.8361536794853947</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>0.9999999999999998</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2149,16 +2204,16 @@
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>0.1313877159362955</v>
+        <v>0.1302869952734138</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>0.07584840651116576</v>
+        <v>0.07511044800018518</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>0.008092723901427012</v>
+        <v>0.007549155191744372</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>0.06641304739379916</v>
+        <v>0.06531094564424378</v>
       </c>
     </row>
     <row r="3">
@@ -2168,16 +2223,16 @@
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>0.1945314254699106</v>
+        <v>0.1933687562137414</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>0.1320994753062168</v>
+        <v>0.1313229433680692</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>0.07354814028538437</v>
+        <v>0.07296901412435819</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>0.1419093586387135</v>
+        <v>0.1407284531935675</v>
       </c>
     </row>
     <row r="4">
@@ -2187,16 +2242,16 @@
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>0.2239917043732078</v>
+        <v>0.2228013084703142</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>0.1538381139497933</v>
+        <v>0.1530475134309137</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>0.08627485542479829</v>
+        <v>0.08568948583438862</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>0.1441318869507096</v>
+        <v>0.1429502946138259</v>
       </c>
     </row>
     <row r="5">
@@ -2206,16 +2261,16 @@
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.2820747786675974</v>
+        <v>0.2808263551231407</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>0.1873015076330251</v>
+        <v>0.1864878886273584</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>0.1145384808719019</v>
+        <v>0.1139376712587177</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.1801426052743265</v>
+        <v>0.1789230182134438</v>
       </c>
     </row>
     <row r="6">
@@ -2225,16 +2280,16 @@
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.2972981334590807</v>
+        <v>0.2960365429272604</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>0.1987020019025265</v>
+        <v>0.1978814543829246</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>0.1163551040103545</v>
+        <v>0.1157539809106296</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>0.1602735866282499</v>
+        <v>0.1590760014186117</v>
       </c>
     </row>
     <row r="7">
@@ -2263,10 +2318,10 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.1477924094523611</v>
+        <v>0.1481610484260478</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>0.0882627916816785</v>
+        <v>0.08807488089967253</v>
       </c>
       <c r="D8" s="1" t="n">
         <v>0.1923053217420418</v>
@@ -2281,6 +2336,348 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Nasdaq-100</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>1. Montant fixe</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>2. Système actuel</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>3. + stratégie 13</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>4. + pilotage du risque</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>5. Les deux</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>SG Trend (vrais fonds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Juil.–oct. 1990 (guerre du Golfe)</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>-0.1917910077826804</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>-0.328966609797709</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>0.6012766253795963</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>0.4500605233778161</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>0.3847837209114271</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>0.4826779308848697</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>0.4251955527407674</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Juil.–août 1998 (Russie, LTCM)</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>-0.1918579958527992</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>-0.2210632731545042</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0.2791809695239531</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>0.202337897777807</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>0.2190055632921857</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>0.2008551774140437</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>0.2177092044082418</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Mars 2000–oct. 2002 (bulle internet)</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>-0.4737718765422733</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>-0.8279012961435407</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>1.020219461367722</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>1.061334718678789</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>1.392848987357972</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>1.703828668391432</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>2.146093355969375</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>0.5333059148312804</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Oct. 2007–mars 2009 (crise financière)</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>-0.5525024213025588</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>-0.5155510494827967</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>1.36921340655889</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>1.385112366642492</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>1.299236587573861</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>1.159977396449488</v>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>1.105729641109479</v>
+      </c>
+      <c r="I5" s="1" t="n">
+        <v>0.3210880351930194</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Avr.–oct. 2011 (crise de l'euro)</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>-0.186407084865727</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>-0.1308449525017542</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>-0.1014469527995864</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>-0.04566364330974948</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>-0.09403545748628672</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>-0.002972032759310572</v>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>-0.04636861383159219</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>-0.04976135664897585</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sept.–déc. 2018</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>-0.1936348952149547</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>-0.2195269376397069</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>0.05558335586001584</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>0.0443123782645769</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>0.05858090500489355</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>0.02887550724094257</v>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>0.04585196888592868</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>-0.03320852494325766</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Févr.–mars 2020 (Covid)</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>-0.3379046158626986</v>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>-0.279164874897979</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>0.4576029657345326</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>0.2862462469941236</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>0.3020742288509728</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>0.3658132485157035</v>
+      </c>
+      <c r="H8" s="1" t="n">
+        <v>0.3050605211165154</v>
+      </c>
+      <c r="I8" s="1" t="n">
+        <v>-0.02438602324765016</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Janv.–oct. 2022 (inflation, taux)</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>-0.2449156252487469</v>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>-0.3428512873062641</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>0.6044064163235694</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>0.4662916276575253</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>0.3615394713010986</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>0.5513344277381786</v>
+      </c>
+      <c r="H9" s="1" t="n">
+        <v>0.4480236836112499</v>
+      </c>
+      <c r="I9" s="1" t="n">
+        <v>0.3564174426952091</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Févr.–avr. 2025 (droits de douane)</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>-0.1874717807894716</v>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>-0.2276831110180648</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>-0.06377414400290271</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>-0.07099797491559667</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>-0.07818172751117225</v>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>-0.1322928694378868</v>
+      </c>
+      <c r="H10" s="1" t="n">
+        <v>-0.1343465763374191</v>
+      </c>
+      <c r="I10" s="1" t="n">
+        <v>-0.1076167764983559</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2341,16 +2738,16 @@
         <v>1990</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>0.3364107449440541</v>
+        <v>0.3328265589004371</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>0.5588616408598253</v>
+        <v>0.5546382933674576</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>0.6204912582161739</v>
+        <v>0.6160904492054917</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>0.7158042013283801</v>
+        <v>0.7111998018952796</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>-0.03104820642576656</v>
@@ -2359,7 +2756,7 @@
         <v>-0.1041168718028905</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>0.08066065701536451</v>
+        <v>0.07774330018656528</v>
       </c>
     </row>
     <row r="3">
@@ -2367,16 +2764,16 @@
         <v>1991</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>0.1737764414737857</v>
+        <v>0.1716034050050712</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>0.2771521932196905</v>
+        <v>0.2747572811494403</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>0.3129285442815684</v>
+        <v>0.3104740795481991</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>0.42985247461127</v>
+        <v>0.4271673153147306</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>0.3046541359519082</v>
@@ -2385,7 +2782,7 @@
         <v>0.6499027576921166</v>
       </c>
       <c r="H3" s="1" t="n">
-        <v>0.05721201445324109</v>
+        <v>0.05522869601871561</v>
       </c>
     </row>
     <row r="4">
@@ -2393,16 +2790,16 @@
         <v>1992</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>-0.008196048438099401</v>
+        <v>-0.009451354684143154</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>0.07828325130386626</v>
+        <v>0.0769228683911678</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>0.06928441272967523</v>
+        <v>0.06793326420999346</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>0.2020166884846268</v>
+        <v>0.2004876256698491</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>0.07620457435940065</v>
@@ -2411,7 +2808,7 @@
         <v>0.08864910610388099</v>
       </c>
       <c r="H4" s="1" t="n">
-        <v>0.03629629134989432</v>
+        <v>0.03498745105596668</v>
       </c>
     </row>
     <row r="5">
@@ -2419,16 +2816,16 @@
         <v>1993</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.441631221220681</v>
+        <v>0.4400815926761383</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>0.4930763239691383</v>
+        <v>0.4914671187222661</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>0.5198407257243587</v>
+        <v>0.5182042587284228</v>
       </c>
       <c r="E5" s="1" t="n">
-        <v>0.6037332627505605</v>
+        <v>0.6020100080746835</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>0.1007787980936903</v>
@@ -2437,7 +2834,7 @@
         <v>0.1057650929383522</v>
       </c>
       <c r="H5" s="1" t="n">
-        <v>0.03153108027272067</v>
+        <v>0.03041915291796826</v>
       </c>
     </row>
     <row r="6">
@@ -2445,16 +2842,16 @@
         <v>1994</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.03760844797422047</v>
+        <v>-0.03920732266094762</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>-0.06173708265189859</v>
+        <v>-0.06329325776993311</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>-0.05691361800581674</v>
+        <v>-0.05847700927784483</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>0.04792056015303903</v>
+        <v>0.04617673728024485</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>0.01321717705033376</v>
@@ -2463,7 +2860,7 @@
         <v>0.01503967058350941</v>
       </c>
       <c r="H6" s="1" t="n">
-        <v>0.04487427789095033</v>
+        <v>0.0431516380936352</v>
       </c>
     </row>
     <row r="7">
@@ -2471,16 +2868,16 @@
         <v>1995</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.3119031034858475</v>
+        <v>0.3094649722868377</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>0.2956746916858277</v>
+        <v>0.293264139484811</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>0.3636873730847578</v>
+        <v>0.3611546875193223</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>0.4288554629806118</v>
+        <v>0.4261878552996419</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>0.3757621024474107</v>
@@ -2489,7 +2886,7 @@
         <v>0.4253592895836935</v>
       </c>
       <c r="H7" s="1" t="n">
-        <v>0.05824437772786961</v>
+        <v>0.05626133943275891</v>
       </c>
     </row>
     <row r="8">
@@ -2497,16 +2894,16 @@
         <v>1996</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.2976754872959007</v>
+        <v>0.2955960838206328</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>0.4165966890668786</v>
+        <v>0.414320375249662</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>0.4544282133559778</v>
+        <v>0.4520920353314188</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>0.4603915449369489</v>
+        <v>0.4580533940973424</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>0.2296096156759775</v>
@@ -2515,7 +2912,7 @@
         <v>0.425403050865109</v>
       </c>
       <c r="H8" s="1" t="n">
-        <v>0.05341377012322024</v>
+        <v>0.05173015370225587</v>
       </c>
     </row>
     <row r="9">
@@ -2523,16 +2920,16 @@
         <v>1997</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.1608272378456002</v>
+        <v>0.1587101811021678</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>0.1878860120718169</v>
+        <v>0.1857175794634764</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>0.2115421437072371</v>
+        <v>0.209334660319896</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>0.3707185322493673</v>
+        <v>0.3681984028758649</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>0.3336276825136044</v>
@@ -2541,7 +2938,7 @@
         <v>0.2063285282945373</v>
       </c>
       <c r="H9" s="1" t="n">
-        <v>0.0538351146071645</v>
+        <v>0.05190586990263535</v>
       </c>
     </row>
     <row r="10">
@@ -2549,16 +2946,16 @@
         <v>1998</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.5042784387243082</v>
+        <v>0.5016251028455569</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>0.6454491344783202</v>
+        <v>0.6425365884404601</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>0.6844145378175359</v>
+        <v>0.6814382407751749</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>0.5988847000648729</v>
+        <v>0.5960793424986763</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>0.2857901787776596</v>
@@ -2567,7 +2964,7 @@
         <v>0.8530020286022797</v>
       </c>
       <c r="H10" s="1" t="n">
-        <v>0.05068894219075948</v>
+        <v>0.048890086721052</v>
       </c>
     </row>
     <row r="11">
@@ -2575,25 +2972,25 @@
         <v>1999</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.1133356419858187</v>
+        <v>0.1114108173942376</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>0.1015388436211275</v>
+        <v>0.09964187527915058</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>0.09334332688647207</v>
+        <v>0.09145956204068395</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>0.08442217417005526</v>
+        <v>0.08255573466084387</v>
       </c>
       <c r="F11" s="1" t="n">
         <v>0.210411913701116</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>0.986838583091173</v>
+        <v>1.019504251066171</v>
       </c>
       <c r="H11" s="1" t="n">
-        <v>0.04924135334993696</v>
+        <v>0.04743737511732715</v>
       </c>
     </row>
     <row r="12">
@@ -2601,25 +2998,25 @@
         <v>2000</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.3100125590477325</v>
+        <v>0.3073003295706214</v>
       </c>
       <c r="C12" s="1" t="n">
-        <v>0.5221348084649471</v>
+        <v>0.5189920232108776</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>0.5768801270898911</v>
+        <v>0.5736279345367357</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>0.3976136369217216</v>
+        <v>0.3947481444613861</v>
       </c>
       <c r="F12" s="1" t="n">
         <v>-0.09104086276837975</v>
       </c>
       <c r="G12" s="1" t="n">
-        <v>-0.3611491036928773</v>
+        <v>-0.3684446158534768</v>
       </c>
       <c r="H12" s="1" t="n">
-        <v>0.06183297271042232</v>
+        <v>0.05964987851852044</v>
       </c>
     </row>
     <row r="13">
@@ -2627,25 +3024,25 @@
         <v>2001</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.1823799187811512</v>
+        <v>0.181320496496356</v>
       </c>
       <c r="C13" s="1" t="n">
-        <v>0.3270872812950412</v>
+        <v>0.3259062382640174</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>0.4022610454797861</v>
+        <v>0.4010159976600323</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>0.1791239794652892</v>
+        <v>0.1780640351720322</v>
       </c>
       <c r="F13" s="1" t="n">
         <v>-0.1188601098308978</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>-0.3334472990133833</v>
+        <v>-0.3265362770636708</v>
       </c>
       <c r="H13" s="1" t="n">
-        <v>0.03582948491767279</v>
+        <v>0.03490918866214732</v>
       </c>
     </row>
     <row r="14">
@@ -2653,25 +3050,25 @@
         <v>2002</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.2481940731148682</v>
+        <v>0.2474781614830803</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>0.333704617947794</v>
+        <v>0.332940420143585</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>0.3650295934024246</v>
+        <v>0.3642504090475009</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>0.3048596895651177</v>
+        <v>0.3041111360237019</v>
       </c>
       <c r="F14" s="1" t="n">
         <v>-0.221003347786878</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>-0.3736840819716171</v>
+        <v>-0.3758156050854439</v>
       </c>
       <c r="H14" s="1" t="n">
-        <v>0.01673679128194716</v>
+        <v>0.01615418449548889</v>
       </c>
     </row>
     <row r="15">
@@ -2679,16 +3076,16 @@
         <v>2003</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.2874460813640747</v>
+        <v>0.2869731882979423</v>
       </c>
       <c r="C15" s="1" t="n">
-        <v>0.3940241042523176</v>
+        <v>0.3935151763744527</v>
       </c>
       <c r="D15" s="1" t="n">
-        <v>0.4431129180477287</v>
+        <v>0.4425859670737535</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>0.332681997545742</v>
+        <v>0.3321926367712649</v>
       </c>
       <c r="F15" s="1" t="n">
         <v>0.2868424808512648</v>
@@ -2697,7 +3094,7 @@
         <v>0.4966900007799731</v>
       </c>
       <c r="H15" s="1" t="n">
-        <v>0.0105025730043975</v>
+        <v>0.01013071119385645</v>
       </c>
     </row>
     <row r="16">
@@ -2705,16 +3102,16 @@
         <v>2004</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.168885554222661</v>
+        <v>0.1681762711650048</v>
       </c>
       <c r="C16" s="1" t="n">
-        <v>0.2547337761735757</v>
+        <v>0.2539761761393784</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>0.2679340660451692</v>
+        <v>0.2671673460094206</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>0.1820792095113621</v>
+        <v>0.1813631399632034</v>
       </c>
       <c r="F16" s="1" t="n">
         <v>0.1088210285038285</v>
@@ -2723,7 +3120,7 @@
         <v>0.1053855549222371</v>
       </c>
       <c r="H16" s="1" t="n">
-        <v>0.0144079319202326</v>
+        <v>0.01379041498544464</v>
       </c>
     </row>
     <row r="17">
@@ -2731,16 +3128,16 @@
         <v>2005</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.05054814523014795</v>
+        <v>0.04926537013177801</v>
       </c>
       <c r="C17" s="1" t="n">
-        <v>0.09271193711141623</v>
+        <v>0.09138312748487132</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>0.09440467063217506</v>
+        <v>0.09307372085556653</v>
       </c>
       <c r="E17" s="1" t="n">
-        <v>0.06045208096850119</v>
+        <v>0.05915740944400527</v>
       </c>
       <c r="F17" s="1" t="n">
         <v>0.04911783501431088</v>
@@ -2749,7 +3146,7 @@
         <v>0.01565202530489662</v>
       </c>
       <c r="H17" s="1" t="n">
-        <v>0.0330526457999103</v>
+        <v>0.0317920801504874</v>
       </c>
     </row>
     <row r="18">
@@ -2757,16 +3154,16 @@
         <v>2006</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.1784356567387302</v>
+        <v>0.1764236032779918</v>
       </c>
       <c r="C18" s="1" t="n">
-        <v>0.1007930320984476</v>
+        <v>0.09890448027665411</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>0.1156148938830504</v>
+        <v>0.1136961743829847</v>
       </c>
       <c r="E18" s="1" t="n">
-        <v>0.1449555235191362</v>
+        <v>0.1430019975132018</v>
       </c>
       <c r="F18" s="1" t="n">
         <v>0.157944638071126</v>
@@ -2775,7 +3172,7 @@
         <v>0.07144328431386748</v>
       </c>
       <c r="H18" s="1" t="n">
-        <v>0.04996968189242024</v>
+        <v>0.04818327970600866</v>
       </c>
     </row>
     <row r="19">
@@ -2783,16 +3180,16 @@
         <v>2007</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.1548949295835453</v>
+        <v>0.1533695262211561</v>
       </c>
       <c r="C19" s="1" t="n">
-        <v>0.07658191051440588</v>
+        <v>0.07515279778111772</v>
       </c>
       <c r="D19" s="1" t="n">
-        <v>0.1075152591002175</v>
+        <v>0.1060505408983301</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>0.1369601273053236</v>
+        <v>0.1354699759382934</v>
       </c>
       <c r="F19" s="1" t="n">
         <v>0.05493726356621176</v>
@@ -2801,7 +3198,7 @@
         <v>0.1902799476875014</v>
       </c>
       <c r="H19" s="1" t="n">
-        <v>0.04613036596297992</v>
+        <v>0.04475014514205888</v>
       </c>
     </row>
     <row r="20">
@@ -2809,16 +3206,16 @@
         <v>2008</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.8937972559428542</v>
+        <v>0.8929097751337944</v>
       </c>
       <c r="C20" s="1" t="n">
-        <v>0.7401204838897604</v>
+        <v>0.7392977998332035</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>0.6650784415087951</v>
+        <v>0.6642918524348846</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>1.06365544316022</v>
+        <v>1.062693446516214</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>-0.3699761081938914</v>
@@ -2827,7 +3224,7 @@
         <v>-0.4172723405513733</v>
       </c>
       <c r="H20" s="1" t="n">
-        <v>0.01434585314311354</v>
+        <v>0.01387279554442689</v>
       </c>
     </row>
     <row r="21">
@@ -2835,16 +3232,16 @@
         <v>2009</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.1300414948563049</v>
+        <v>-0.1301067482538147</v>
       </c>
       <c r="C21" s="1" t="n">
-        <v>-0.08684241920752656</v>
+        <v>-0.08691090048910433</v>
       </c>
       <c r="D21" s="1" t="n">
-        <v>-0.04712304146026913</v>
+        <v>-0.04719440910137129</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>-0.1386620011560769</v>
+        <v>-0.1387263635251382</v>
       </c>
       <c r="F21" s="1" t="n">
         <v>0.264642321298298</v>
@@ -2853,7 +3250,7 @@
         <v>0.5468432209179339</v>
       </c>
       <c r="H21" s="1" t="n">
-        <v>0.001551196248863462</v>
+        <v>0.001476973522390512</v>
       </c>
     </row>
     <row r="22">
@@ -2861,16 +3258,16 @@
         <v>2010</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.2328177977828407</v>
+        <v>0.2327397095361299</v>
       </c>
       <c r="C22" s="1" t="n">
-        <v>0.2892720636040027</v>
+        <v>0.2891907163221452</v>
       </c>
       <c r="D22" s="1" t="n">
-        <v>0.2945720987479739</v>
+        <v>0.2944902503949314</v>
       </c>
       <c r="E22" s="1" t="n">
-        <v>0.2401055525335773</v>
+        <v>0.2400270847746733</v>
       </c>
       <c r="F22" s="1" t="n">
         <v>0.15063401360544</v>
@@ -2879,7 +3276,7 @@
         <v>0.2014364886282187</v>
       </c>
       <c r="H22" s="1" t="n">
-        <v>0.001429190828477145</v>
+        <v>0.001366681595040609</v>
       </c>
     </row>
     <row r="23">
@@ -2887,16 +3284,16 @@
         <v>2011</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.009438625265494216</v>
+        <v>-0.009457972953615279</v>
       </c>
       <c r="C23" s="1" t="n">
-        <v>0.08305621096612037</v>
+        <v>0.08303503399331325</v>
       </c>
       <c r="D23" s="1" t="n">
-        <v>0.09979360456284381</v>
+        <v>0.09977210961041982</v>
       </c>
       <c r="E23" s="1" t="n">
-        <v>-0.04065362649377169</v>
+        <v>-0.04067232355934247</v>
       </c>
       <c r="F23" s="1" t="n">
         <v>0.02111820043608126</v>
@@ -2905,7 +3302,7 @@
         <v>0.03475807772937101</v>
       </c>
       <c r="H23" s="1" t="n">
-        <v>0.0005422094031992675</v>
+        <v>0.0005228751307688739</v>
       </c>
     </row>
     <row r="24">
@@ -2913,16 +3310,16 @@
         <v>2012</v>
       </c>
       <c r="B24" s="1" t="n">
-        <v>-0.117912724973108</v>
+        <v>-0.1179488931217455</v>
       </c>
       <c r="C24" s="1" t="n">
-        <v>-0.05180629410004522</v>
+        <v>-0.05184523659744611</v>
       </c>
       <c r="D24" s="1" t="n">
-        <v>-0.08547141272699221</v>
+        <v>-0.08550894784433116</v>
       </c>
       <c r="E24" s="1" t="n">
-        <v>-0.1167338140742247</v>
+        <v>-0.1167700130276567</v>
       </c>
       <c r="F24" s="1" t="n">
         <v>0.1600322380427452</v>
@@ -2931,7 +3328,7 @@
         <v>0.1811253955977239</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>0.0009055668352333512</v>
+        <v>0.0008644810626574628</v>
       </c>
     </row>
     <row r="25">
@@ -2939,16 +3336,16 @@
         <v>2013</v>
       </c>
       <c r="B25" s="1" t="n">
-        <v>-0.01006657202662442</v>
+        <v>-0.01009236002720015</v>
       </c>
       <c r="C25" s="1" t="n">
-        <v>0.0262197125240673</v>
+        <v>0.02619291931603307</v>
       </c>
       <c r="D25" s="1" t="n">
-        <v>0.02599103981817552</v>
+        <v>0.02596422280967348</v>
       </c>
       <c r="E25" s="1" t="n">
-        <v>0.03692192361804514</v>
+        <v>0.03689491476386597</v>
       </c>
       <c r="F25" s="1" t="n">
         <v>0.3238847806296004</v>
@@ -2957,7 +3354,7 @@
         <v>0.3663422322212719</v>
       </c>
       <c r="H25" s="1" t="n">
-        <v>0.0005942232934741387</v>
+        <v>0.0005681055567328119</v>
       </c>
     </row>
     <row r="26">
@@ -2965,16 +3362,16 @@
         <v>2014</v>
       </c>
       <c r="B26" s="1" t="n">
-        <v>0.5241849131968894</v>
+        <v>0.5241609765401987</v>
       </c>
       <c r="C26" s="1" t="n">
-        <v>0.5515309777344697</v>
+        <v>0.5515066209373949</v>
       </c>
       <c r="D26" s="1" t="n">
-        <v>0.6204400143736439</v>
+        <v>0.6204146040906384</v>
       </c>
       <c r="E26" s="1" t="n">
-        <v>0.5347330811945783</v>
+        <v>0.5347089734709158</v>
       </c>
       <c r="F26" s="1" t="n">
         <v>0.1368836315708499</v>
@@ -2983,7 +3380,7 @@
         <v>0.1918141645796192</v>
       </c>
       <c r="H26" s="1" t="n">
-        <v>0.0003369612625909735</v>
+        <v>0.0003211471355331064</v>
       </c>
     </row>
     <row r="27">
@@ -2991,16 +3388,16 @@
         <v>2015</v>
       </c>
       <c r="B27" s="1" t="n">
-        <v>0.05249251677825217</v>
+        <v>0.05244768643511466</v>
       </c>
       <c r="C27" s="1" t="n">
-        <v>0.06204158283961658</v>
+        <v>0.06199645497259243</v>
       </c>
       <c r="D27" s="1" t="n">
-        <v>0.09148851789984791</v>
+        <v>0.09144209486857635</v>
       </c>
       <c r="E27" s="1" t="n">
-        <v>0.004133177421054013</v>
+        <v>0.004090367647606064</v>
       </c>
       <c r="F27" s="1" t="n">
         <v>0.01383759921898431</v>
@@ -3009,7 +3406,7 @@
         <v>0.09435423949203803</v>
       </c>
       <c r="H27" s="1" t="n">
-        <v>0.000544591224157509</v>
+        <v>0.0005025904769846434</v>
       </c>
     </row>
     <row r="28">
@@ -3017,16 +3414,16 @@
         <v>2016</v>
       </c>
       <c r="B28" s="1" t="n">
-        <v>-0.06364167197724568</v>
+        <v>-0.06378496541728684</v>
       </c>
       <c r="C28" s="1" t="n">
-        <v>-0.05029026300721728</v>
+        <v>-0.05043609258734705</v>
       </c>
       <c r="D28" s="1" t="n">
-        <v>-0.06341950971195687</v>
+        <v>-0.06356330227457485</v>
       </c>
       <c r="E28" s="1" t="n">
-        <v>-0.1072347408268292</v>
+        <v>-0.107371685095662</v>
       </c>
       <c r="F28" s="1" t="n">
         <v>0.1195991207871063</v>
@@ -3035,7 +3432,7 @@
         <v>0.07098286188239489</v>
       </c>
       <c r="H28" s="1" t="n">
-        <v>0.003287114685658787</v>
+        <v>0.003133640586880038</v>
       </c>
     </row>
     <row r="29">
@@ -3043,16 +3440,16 @@
         <v>2017</v>
       </c>
       <c r="B29" s="1" t="n">
-        <v>-0.06933580687453911</v>
+        <v>-0.06970002493193372</v>
       </c>
       <c r="C29" s="1" t="n">
-        <v>0.01039582389401139</v>
+        <v>0.009999733443356584</v>
       </c>
       <c r="D29" s="1" t="n">
-        <v>0.01279583961883901</v>
+        <v>0.01239878062233202</v>
       </c>
       <c r="E29" s="1" t="n">
-        <v>-0.07921420012731761</v>
+        <v>-0.07957347839765949</v>
       </c>
       <c r="F29" s="1" t="n">
         <v>0.2183160148270713</v>
@@ -3061,7 +3458,7 @@
         <v>0.326636469242753</v>
       </c>
       <c r="H29" s="1" t="n">
-        <v>0.009667671520190435</v>
+        <v>0.009272910567206916</v>
       </c>
     </row>
     <row r="30">
@@ -3069,16 +3466,16 @@
         <v>2018</v>
       </c>
       <c r="B30" s="1" t="n">
-        <v>-0.03885591189532767</v>
+        <v>-0.0394927454120757</v>
       </c>
       <c r="C30" s="1" t="n">
-        <v>-0.01012306645161087</v>
+        <v>-0.01077791204280565</v>
       </c>
       <c r="D30" s="1" t="n">
-        <v>-0.0008089690704168317</v>
+        <v>-0.001470328528414888</v>
       </c>
       <c r="E30" s="1" t="n">
-        <v>-0.05437841152766099</v>
+        <v>-0.05501063281388485</v>
       </c>
       <c r="F30" s="1" t="n">
         <v>-0.0438424174525569</v>
@@ -3087,7 +3484,7 @@
         <v>-0.001262566267758447</v>
       </c>
       <c r="H30" s="1" t="n">
-        <v>0.02027017051082791</v>
+        <v>0.01959148166144886</v>
       </c>
     </row>
     <row r="31">
@@ -3095,16 +3492,16 @@
         <v>2019</v>
       </c>
       <c r="B31" s="1" t="n">
-        <v>0.00511539006151196</v>
+        <v>0.004375368811789349</v>
       </c>
       <c r="C31" s="1" t="n">
-        <v>0.05863439417753558</v>
+        <v>0.05785373687071838</v>
       </c>
       <c r="D31" s="1" t="n">
-        <v>0.1191566938451318</v>
+        <v>0.1183328409738975</v>
       </c>
       <c r="E31" s="1" t="n">
-        <v>0.04115978304755186</v>
+        <v>0.04038548564085676</v>
       </c>
       <c r="F31" s="1" t="n">
         <v>0.3148637098683436</v>
@@ -3113,7 +3510,7 @@
         <v>0.389613478961214</v>
       </c>
       <c r="H31" s="1" t="n">
-        <v>0.02157173616791308</v>
+        <v>0.02081335978505661</v>
       </c>
     </row>
     <row r="32">
@@ -3121,16 +3518,16 @@
         <v>2020</v>
       </c>
       <c r="B32" s="1" t="n">
-        <v>0.2689819175695285</v>
+        <v>0.2688503199566659</v>
       </c>
       <c r="C32" s="1" t="n">
-        <v>0.18553685610764</v>
+        <v>0.1854159240470687</v>
       </c>
       <c r="D32" s="1" t="n">
-        <v>0.261848913812428</v>
+        <v>0.2617207514397037</v>
       </c>
       <c r="E32" s="1" t="n">
-        <v>0.3849911090164657</v>
+        <v>0.3848448605666992</v>
       </c>
       <c r="F32" s="1" t="n">
         <v>0.1839882689892662</v>
@@ -3139,7 +3536,7 @@
         <v>0.4840651869821666</v>
       </c>
       <c r="H32" s="1" t="n">
-        <v>0.003762532532923579</v>
+        <v>0.003658352876944715</v>
       </c>
     </row>
     <row r="33">
@@ -3147,16 +3544,16 @@
         <v>2021</v>
       </c>
       <c r="B33" s="1" t="n">
-        <v>0.1688166779198979</v>
+        <v>0.1687968922891316</v>
       </c>
       <c r="C33" s="1" t="n">
-        <v>0.1051639887328095</v>
+        <v>0.1051453002216469</v>
       </c>
       <c r="D33" s="1" t="n">
-        <v>0.1106116067023808</v>
+        <v>0.1105927977176304</v>
       </c>
       <c r="E33" s="1" t="n">
-        <v>0.3765243948322559</v>
+        <v>0.3765011220791668</v>
       </c>
       <c r="F33" s="1" t="n">
         <v>0.2870536836204058</v>
@@ -3165,7 +3562,7 @@
         <v>0.2741959404012131</v>
       </c>
       <c r="H33" s="1" t="n">
-        <v>0.0004711421957845907</v>
+        <v>0.0004543491391522103</v>
       </c>
     </row>
     <row r="34">
@@ -3173,16 +3570,16 @@
         <v>2022</v>
       </c>
       <c r="B34" s="1" t="n">
-        <v>0.2292563157667264</v>
+        <v>0.2279588126474139</v>
       </c>
       <c r="C34" s="1" t="n">
-        <v>0.1527789758183404</v>
+        <v>0.1515619260162155</v>
       </c>
       <c r="D34" s="1" t="n">
-        <v>0.1325405190941553</v>
+        <v>0.1313460265959532</v>
       </c>
       <c r="E34" s="1" t="n">
-        <v>0.2871688057845152</v>
+        <v>0.2858102521909065</v>
       </c>
       <c r="F34" s="1" t="n">
         <v>-0.181108874803489</v>
@@ -3191,7 +3588,7 @@
         <v>-0.3257705080852904</v>
       </c>
       <c r="H34" s="1" t="n">
-        <v>0.02118912856690836</v>
+        <v>0.02011425446538673</v>
       </c>
     </row>
     <row r="35">
@@ -3199,16 +3596,16 @@
         <v>2023</v>
       </c>
       <c r="B35" s="1" t="n">
-        <v>-0.0136872381728903</v>
+        <v>-0.01548812861315541</v>
       </c>
       <c r="C35" s="1" t="n">
-        <v>0.06046240287543547</v>
+        <v>0.05851543001097492</v>
       </c>
       <c r="D35" s="1" t="n">
-        <v>0.07723577165079232</v>
+        <v>0.07525881626066333</v>
       </c>
       <c r="E35" s="1" t="n">
-        <v>-0.03890059286396619</v>
+        <v>-0.0406513510796106</v>
       </c>
       <c r="F35" s="1" t="n">
         <v>0.2628729203401294</v>
@@ -3217,7 +3614,7 @@
         <v>0.5485583636391509</v>
       </c>
       <c r="H35" s="1" t="n">
-        <v>0.05368206288261623</v>
+        <v>0.05174363544728533</v>
       </c>
     </row>
     <row r="36">
@@ -3227,16 +3624,16 @@
         </is>
       </c>
       <c r="B36" s="1" t="n">
-        <v>0.0868513652002818</v>
+        <v>0.08642517331258803</v>
       </c>
       <c r="C36" s="1" t="n">
-        <v>0.1131157685155364</v>
+        <v>0.1126797409754272</v>
       </c>
       <c r="D36" s="1" t="n">
-        <v>0.1286170820159536</v>
+        <v>0.1281750386041882</v>
       </c>
       <c r="E36" s="1" t="n">
-        <v>0.05247776958923978</v>
+        <v>0.05206621958994551</v>
       </c>
       <c r="F36" s="1" t="n">
         <v>0.1055597513507232</v>
@@ -3245,7 +3642,7 @@
         <v>0.08565369904278763</v>
       </c>
       <c r="H36" s="1" t="n">
-        <v>0.01337819093538717</v>
+        <v>0.0129843133949572</v>
       </c>
     </row>
   </sheetData>
@@ -3253,13 +3650,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3309,23 +3706,23 @@
           <t>CAGR (rendement total)</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>0.1547230517396851</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>0.1962903790563373</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>0.2167605669438251</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>0.2103026884966808</v>
-      </c>
-      <c r="F2" s="2" t="n">
+      <c r="B2" s="1" t="n">
+        <v>0.1536379941288943</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>0.1951641421712746</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>0.2156157117884818</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>0.2091647585464489</v>
+      </c>
+      <c r="F2" s="1" t="n">
         <v>0.1045428525236882</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>0.1414968884518983</v>
+      <c r="G2" s="1" t="n">
+        <v>0.1418879597940064</v>
       </c>
     </row>
     <row r="3">
@@ -3334,23 +3731,23 @@
           <t>CAGR au même risque que le S&amp;P 500</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>0.1534498143118921</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>0.2141459825153116</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>0.2316701415058011</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>0.2110334943155077</v>
-      </c>
-      <c r="F3" s="2" t="n">
+      <c r="B3" s="1" t="n">
+        <v>0.1523607528187074</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>0.212994241034882</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0.2305017804893581</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>0.2098867066044021</v>
+      </c>
+      <c r="F3" s="1" t="n">
         <v>0.1045428525236882</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>0.1130057687257837</v>
+      <c r="G3" s="1" t="n">
+        <v>0.1127137099510904</v>
       </c>
     </row>
     <row r="4">
@@ -3359,23 +3756,23 @@
           <t>Volatilité annualisée (écart-type quotidien)</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>0.1815915393670031</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>0.1620879010447896</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>0.1664150983715982</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>0.1788698450367996</v>
-      </c>
-      <c r="F4" s="2" t="n">
+      <c r="B4" s="1" t="n">
+        <v>0.1816018376607463</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>0.1621109457875019</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>0.1664344881103929</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>0.1788844832287072</v>
+      </c>
+      <c r="F4" s="1" t="n">
         <v>0.1795720672483162</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>0.2605168478834615</v>
+      <c r="G4" s="1" t="n">
+        <v>0.2615530119752032</v>
       </c>
     </row>
     <row r="5">
@@ -3384,322 +3781,348 @@
           <t>Écart-type des performances annuelles</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>0.2143629335556832</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>0.2204405719930536</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>0.2304912779378683</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>0.2732339467038686</v>
-      </c>
-      <c r="F5" s="2" t="n">
+      <c r="B5" s="1" t="n">
+        <v>0.2140595157669709</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>0.219956955790629</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0.2299661267826774</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>0.2727022537328466</v>
+      </c>
+      <c r="F5" s="1" t="n">
         <v>0.1766370522118561</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>0.3362368238542294</v>
+      <c r="G5" s="1" t="n">
+        <v>0.3387718183977626</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sharpe</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>0.721649625747524</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>1.002009138477459</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>1.080388657333119</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>0.9880507622765542</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>0.4848480348960219</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>0.5263253135556422</v>
-      </c>
+          <t>Exposition moyenne (notionnel / capital)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sortino</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>1.024159709135418</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>1.447077341750245</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>1.560741035495825</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>1.410151414797085</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>0.6851541757999026</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>0.7556477717213654</v>
-      </c>
+          <t>Coûts par an (transactions + roulement)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Calmar (CAGR / pire baisse)</t>
+          <t>Sharpe</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.4485202921850494</v>
+        <v>0.721649625747524</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.7337363049620097</v>
+        <v>1.002009138477459</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.8472605686673254</v>
+        <v>1.080388657333119</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.5236370159508984</v>
+        <v>0.9880507622765542</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.1892170033883688</v>
+        <v>0.4899846961673663</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.1705524185156602</v>
+        <v>0.5299776412362787</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pire baisse (max drawdown)</t>
+          <t>Sortino</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>-0.3449633259309701</v>
+        <v>1.024159709135418</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.2675216937323287</v>
+        <v>1.447077341750245</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>-0.2558369584988152</v>
+        <v>1.560741035495825</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-0.4016192173022407</v>
+        <v>1.410151414797085</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-0.5525024213025587</v>
+        <v>0.6926260522270149</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>-0.8296387098076012</v>
+        <v>0.7636683740978054</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Meilleure année</t>
+          <t>Calmar (CAGR / pire baisse)</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.8937972559428542</v>
+        <v>0.4443937682326982</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.7401204838897604</v>
+        <v>0.7293973510158117</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.6844145378175359</v>
+        <v>0.8415178579139589</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>1.06365544316022</v>
+        <v>0.5199008575500947</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.3757621024474107</v>
+        <v>0.1892170033883688</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.986838583091173</v>
+        <v>0.1711613170674666</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Pire année</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>-0.1300414948563049</v>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>-0.08684241920752656</v>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>-0.08547141272699221</v>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>-0.1386620011560769</v>
-      </c>
-      <c r="F11" s="2" t="n">
-        <v>-0.3699761081938914</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>-0.4172723405513733</v>
+          <t>Pire baisse (max drawdown)</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>-0.3457249068543301</v>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>-0.267569030651777</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>-0.2562223840655886</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>-0.4023166253890915</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>-0.5525024213025587</v>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>-0.8289721195477741</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Années positives</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>0.7058823529411765</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>0.8529411764705882</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>0.8529411764705882</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>0.7941176470588235</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>0.7941176470588235</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>0.7941176470588235</v>
+          <t>Meilleure année</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>0.8929097751337944</v>
+      </c>
+      <c r="C12" s="1" t="n">
+        <v>0.7392977998332035</v>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>0.6814382407751749</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>1.062693446516214</v>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>0.3757621024474107</v>
+      </c>
+      <c r="G12" s="1" t="n">
+        <v>1.019504251066171</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Pire mois</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>-0.1242879723703741</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>-0.1109193498486285</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>-0.1169769254572505</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>-0.1074379876370939</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>-0.1679506188757092</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>-0.2620526558891454</v>
+          <t>Pire année</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>-0.1301067482538147</v>
+      </c>
+      <c r="C13" s="1" t="n">
+        <v>-0.08691090048910433</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>-0.08550894784433116</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>-0.1387263635251382</v>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>-0.3699761081938914</v>
+      </c>
+      <c r="G13" s="1" t="n">
+        <v>-0.4172723405513733</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mois positifs</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>0.6009732360097324</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>0.6301703163017032</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>0.6204379562043796</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>0.6228710462287105</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>0.6593673965936739</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>0.6058394160583942</v>
+          <t>Années positives</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>0.7058823529411765</v>
+      </c>
+      <c r="C14" s="1" t="n">
+        <v>0.8529411764705882</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>0.8529411764705882</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>0.7941176470588235</v>
+      </c>
+      <c r="F14" s="1" t="n">
+        <v>0.7941176470588235</v>
+      </c>
+      <c r="G14" s="1" t="n">
+        <v>0.7941176470588235</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Skew mensuel</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>0.5535765412313605</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>0.3805484842273775</v>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>0.2899483348957997</v>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>0.6823868639303342</v>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>-0.5415043213897184</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>-0.2833074562421103</v>
+          <t>Pire mois</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>-0.1243727205182223</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>-0.1111384143786313</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>-0.1170213323282306</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>-0.1075625574043143</v>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>-0.1679506188757092</v>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>-0.2640493636714231</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Corrélation S&amp;P 500 (mensuelle)</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>-0.255215423039872</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>-0.2550267321066124</v>
-      </c>
-      <c r="D16" s="2" t="n">
-        <v>-0.1898382724485805</v>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>-0.2242255440166658</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>0.8332417790525114</v>
+          <t>Mois positifs</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>0.6009732360097324</v>
+      </c>
+      <c r="C16" s="1" t="n">
+        <v>0.6301703163017032</v>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>0.6204379562043796</v>
+      </c>
+      <c r="E16" s="1" t="n">
+        <v>0.6228710462287105</v>
+      </c>
+      <c r="F16" s="1" t="n">
+        <v>0.6593673965936739</v>
+      </c>
+      <c r="G16" s="1" t="n">
+        <v>0.6058394160583942</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Skew mensuel</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>0.5539622109099078</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>0.3799344061671359</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>0.2895853666770165</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>0.6829156125452053</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>-0.5415043213897184</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>-0.2754286005240467</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Corrélation S&amp;P 500 (mensuelle)</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>-0.2552146716058428</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>-0.2550400138964743</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>-0.1898654496764285</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>-0.2241478687441297</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0.8325145799821074</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>Corrélation Nasdaq-100 (mensuelle)</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
-        <v>-0.2275954749997774</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>-0.238758572225619</v>
-      </c>
-      <c r="D17" s="2" t="n">
-        <v>-0.1898443095822149</v>
-      </c>
-      <c r="E17" s="2" t="n">
-        <v>-0.1998792366591489</v>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>0.8332417790525113</v>
-      </c>
-      <c r="G17" s="2" t="n">
+      <c r="B19" s="2" t="n">
+        <v>-0.2279061630274398</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>-0.2394411451710921</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>-0.1906454401176129</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>-0.1998937392032669</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0.8325145799821074</v>
+      </c>
+      <c r="G19" s="2" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>